<commit_message>
Se agregan avances del proyecto (fueron muchos y olvidé subirlos antes)
</commit_message>
<xml_diff>
--- a/Modelo/datos/Intermedias/matriz_sin_redundancia_v2.xlsx
+++ b/Modelo/datos/Intermedias/matriz_sin_redundancia_v2.xlsx
@@ -1,21 +1,248 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21a7d57e8591b932/Escritorio/CICS/2025/Tesis/Objetivos de Aprendizaje/Modelo/datos/Intermedias/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2F6F1ED98F79A8D366075C52F37BD2722A4AE7D1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E40EB462-BFD7-4DFD-A16F-849EE5C30E04}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="19386" windowHeight="11466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="72">
+  <si>
+    <t>Concepto</t>
+  </si>
+  <si>
+    <t>Jubilación</t>
+  </si>
+  <si>
+    <t>Rentabilidad</t>
+  </si>
+  <si>
+    <t>Que_es_pension</t>
+  </si>
+  <si>
+    <t>Pension_Autofinanciada</t>
+  </si>
+  <si>
+    <t>Entidades_Reguladoras</t>
+  </si>
+  <si>
+    <t>AFP</t>
+  </si>
+  <si>
+    <t>Compania_Seguros</t>
+  </si>
+  <si>
+    <t>Diferencia_AFP_CSV</t>
+  </si>
+  <si>
+    <t>Cotizaciones_Previsionales</t>
+  </si>
+  <si>
+    <t>Saldo_Cuenta_Individual</t>
+  </si>
+  <si>
+    <t>Proceso_Solicitud</t>
+  </si>
+  <si>
+    <t>Inicio_Proceso_AFP</t>
+  </si>
+  <si>
+    <t>Formulario_Solicitud_Pension</t>
+  </si>
+  <si>
+    <t>Certificado_de_Saldo</t>
+  </si>
+  <si>
+    <t>Definicion_SCOMP</t>
+  </si>
+  <si>
+    <t>Solicitud_Ofertas</t>
+  </si>
+  <si>
+    <t>Certificado_Oferta</t>
+  </si>
+  <si>
+    <t>Opciones_Post_Oferta</t>
+  </si>
+  <si>
+    <t>Remate</t>
+  </si>
+  <si>
+    <t>Evaluacion_Ofertas</t>
+  </si>
+  <si>
+    <t>Acepta_Rechazo_Oferta</t>
+  </si>
+  <si>
+    <t>Formulario_Seleccion_Modalidad</t>
+  </si>
+  <si>
+    <t>Materializacion_Eleccion</t>
+  </si>
+  <si>
+    <t>Causas_Finalizacion_Proceso</t>
+  </si>
+  <si>
+    <t>Traslado_Fondos</t>
+  </si>
+  <si>
+    <t>Inicio_Pagos</t>
+  </si>
+  <si>
+    <t>Errores_Formularios</t>
+  </si>
+  <si>
+    <t>Demora_Certificados</t>
+  </si>
+  <si>
+    <t>Modalidades_Pensiones</t>
+  </si>
+  <si>
+    <t>Comparacion_modalidades</t>
+  </si>
+  <si>
+    <t>Expectativa_Vida</t>
+  </si>
+  <si>
+    <t>Riesgo_Longevidad</t>
+  </si>
+  <si>
+    <t>Riesgo_Rentabilidad</t>
+  </si>
+  <si>
+    <t>Tasa_Interes_Tecnica_RP</t>
+  </si>
+  <si>
+    <t>Tasa_Interes_RV</t>
+  </si>
+  <si>
+    <t>Cambio_Modalidad</t>
+  </si>
+  <si>
+    <t>Renta_Vitalicia</t>
+  </si>
+  <si>
+    <t>Requisitos_RV</t>
+  </si>
+  <si>
+    <t>Condiciones_Especiales_RV</t>
+  </si>
+  <si>
+    <t>Periodo_Garantizado</t>
+  </si>
+  <si>
+    <t>Clausula_Incremento_Sobrevivencia</t>
+  </si>
+  <si>
+    <t>Aumento_Temporal</t>
+  </si>
+  <si>
+    <t>Calculo_Renta_Vitalicia</t>
+  </si>
+  <si>
+    <t>Retiro_Programado</t>
+  </si>
+  <si>
+    <t>Requisitos_RP</t>
+  </si>
+  <si>
+    <t>Calculo_Retiro_Programado</t>
+  </si>
+  <si>
+    <t>RVI_RP</t>
+  </si>
+  <si>
+    <t>Requisitos_RVI_RP</t>
+  </si>
+  <si>
+    <t>RT_RVD</t>
+  </si>
+  <si>
+    <t>Periodo_Diferimiento</t>
+  </si>
+  <si>
+    <t>Requisitos_RT_RVD</t>
+  </si>
+  <si>
+    <t>Calculo_Rentas_Combinadas</t>
+  </si>
+  <si>
+    <t>Beneficiarios_Legales</t>
+  </si>
+  <si>
+    <t>Declaracion_Beneficiarios</t>
+  </si>
+  <si>
+    <t>Pension_Sobrevivencia</t>
+  </si>
+  <si>
+    <t>Ejemplo_Calculo_Pension_Sobrevivencia</t>
+  </si>
+  <si>
+    <t>Herencia</t>
+  </si>
+  <si>
+    <t>Quien_Recibe_Herencia</t>
+  </si>
+  <si>
+    <t>Como_Calcular_Herencia</t>
+  </si>
+  <si>
+    <t>Definicion_APV</t>
+  </si>
+  <si>
+    <t>Movilidad_Fondos_APV_Pension</t>
+  </si>
+  <si>
+    <t>ELD</t>
+  </si>
+  <si>
+    <t>Calculo_ELD</t>
+  </si>
+  <si>
+    <t>Tratamiento_Tributario_ELD</t>
+  </si>
+  <si>
+    <t>Impacto_Pension_ELD</t>
+  </si>
+  <si>
+    <t>Procedimiento_Retiro_ELD</t>
+  </si>
+  <si>
+    <t>Asesores_Prev</t>
+  </si>
+  <si>
+    <t>Comisiones_AFP</t>
+  </si>
+  <si>
+    <t>Comisiones_Aseguradoras</t>
+  </si>
+  <si>
+    <t>Impacto_Comisiones</t>
+  </si>
+  <si>
+    <t>Falta_Claridad_Comisiones</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,13 +290,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -107,7 +342,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -141,6 +376,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -175,9 +411,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -350,377 +587,234 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BT72"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.9375" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
+  <cols>
+    <col min="1" max="1" width="22.76171875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Jubilación</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Que_es_pension</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Pension_Autofinanciada</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Entidades_Reguladoras</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>AFP</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Compania_Seguros</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Diferencia_AFP_CSV</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Cotizaciones_Previsionales</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Saldo_Cuenta_Individual</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Proceso_Solicitud</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Inicio_Proceso_AFP</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Formulario_Solicitud_Pension</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Certificado_de_Saldo</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Definicion_SCOMP</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Solicitud_Ofertas</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Certificado_Oferta</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Opciones_Post_Oferta</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Remate</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Evaluacion_Ofertas</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Acepta_Rechazo_Oferta</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Formulario_Seleccion_Modalidad</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Materializacion_Eleccion</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Causas_Finalizacion_Proceso</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Traslado_Fondos</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Inicio_Pagos</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>Errores_Formularios</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>Demora_Certificados</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Modalidades_Pensiones</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>Comparacion_modalidades</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>Expectativa_Vida</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>Riesgo_Longevidad</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>Riesgo_Rentabilidad</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>Tasa_Interes_Tecnica_RP</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>Tasa_Interes_RV</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>Cambio_Modalidad</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>Renta_Vitalicia</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>Requisitos_RV</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>Condiciones_Especiales_RV</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>Periodo_Garantizado</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>Clausula_Incremento_Sobrevivencia</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>Aumento_Temporal</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>Calculo_Renta_Vitalicia</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>Retiro_Programado</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>Requisitos_RP</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>Calculo_Retiro_Programado</t>
-        </is>
-      </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>RVI_RP</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>Requisitos_RVI_RP</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>RT_RVD</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
-        <is>
-          <t>Periodo_Diferimiento</t>
-        </is>
-      </c>
-      <c r="AZ1" s="1" t="inlineStr">
-        <is>
-          <t>Requisitos_RT_RVD</t>
-        </is>
-      </c>
-      <c r="BA1" s="1" t="inlineStr">
-        <is>
-          <t>Calculo_Rentas_Combinadas</t>
-        </is>
-      </c>
-      <c r="BB1" s="1" t="inlineStr">
-        <is>
-          <t>Beneficiarios_Legales</t>
-        </is>
-      </c>
-      <c r="BC1" s="1" t="inlineStr">
-        <is>
-          <t>Declaracion_Beneficiarios</t>
-        </is>
-      </c>
-      <c r="BD1" s="1" t="inlineStr">
-        <is>
-          <t>Pension_Sobrevivencia</t>
-        </is>
-      </c>
-      <c r="BE1" s="1" t="inlineStr">
-        <is>
-          <t>Ejemplo_Calculo_Pension_Sobrevivencia</t>
-        </is>
-      </c>
-      <c r="BF1" s="1" t="inlineStr">
-        <is>
-          <t>Herencia</t>
-        </is>
-      </c>
-      <c r="BG1" s="1" t="inlineStr">
-        <is>
-          <t>Quien_Recibe_Herencia</t>
-        </is>
-      </c>
-      <c r="BH1" s="1" t="inlineStr">
-        <is>
-          <t>Como_Calcular_Herencia</t>
-        </is>
-      </c>
-      <c r="BI1" s="1" t="inlineStr">
-        <is>
-          <t>Definicion_APV</t>
-        </is>
-      </c>
-      <c r="BJ1" s="1" t="inlineStr">
-        <is>
-          <t>Movilidad_Fondos_APV_Pension</t>
-        </is>
-      </c>
-      <c r="BK1" s="1" t="inlineStr">
-        <is>
-          <t>ELD</t>
-        </is>
-      </c>
-      <c r="BL1" s="1" t="inlineStr">
-        <is>
-          <t>Calculo_ELD</t>
-        </is>
-      </c>
-      <c r="BM1" s="1" t="inlineStr">
-        <is>
-          <t>Tratamiento_Tributario_ELD</t>
-        </is>
-      </c>
-      <c r="BN1" s="1" t="inlineStr">
-        <is>
-          <t>Impacto_Pension_ELD</t>
-        </is>
-      </c>
-      <c r="BO1" s="1" t="inlineStr">
-        <is>
-          <t>Procedimiento_Retiro_ELD</t>
-        </is>
-      </c>
-      <c r="BP1" s="1" t="inlineStr">
-        <is>
-          <t>Asesores_Prev</t>
-        </is>
-      </c>
-      <c r="BQ1" s="1" t="inlineStr">
-        <is>
-          <t>Comisiones_AFP</t>
-        </is>
-      </c>
-      <c r="BR1" s="1" t="inlineStr">
-        <is>
-          <t>Comisiones_Aseguradoras</t>
-        </is>
-      </c>
-      <c r="BS1" s="1" t="inlineStr">
-        <is>
-          <t>Impacto_Comisiones</t>
-        </is>
-      </c>
-      <c r="BT1" s="1" t="inlineStr">
-        <is>
-          <t>Falta_Claridad_Comisiones</t>
-        </is>
+    <row r="1" spans="1:72" s="1" customFormat="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="BA1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="BB1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="BC1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BD1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="BF1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BG1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="BP1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Jubilación</t>
-        </is>
+    <row r="2" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A2" t="s">
+        <v>1</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -936,11 +1030,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Rentabilidad</t>
-        </is>
+    <row r="3" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A3" t="s">
+        <v>2</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1156,11 +1248,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Que_es_pension</t>
-        </is>
+    <row r="4" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A4" t="s">
+        <v>3</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1376,11 +1466,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Pension_Autofinanciada</t>
-        </is>
+    <row r="5" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A5" t="s">
+        <v>4</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1596,11 +1684,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Entidades_Reguladoras</t>
-        </is>
+    <row r="6" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A6" t="s">
+        <v>5</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1816,11 +1902,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AFP</t>
-        </is>
+    <row r="7" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A7" t="s">
+        <v>6</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2036,11 +2120,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Compania_Seguros</t>
-        </is>
+    <row r="8" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A8" t="s">
+        <v>7</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2256,11 +2338,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Diferencia_AFP_CSV</t>
-        </is>
+    <row r="9" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A9" t="s">
+        <v>8</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2476,11 +2556,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Cotizaciones_Previsionales</t>
-        </is>
+    <row r="10" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A10" t="s">
+        <v>9</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -2696,11 +2774,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Saldo_Cuenta_Individual</t>
-        </is>
+    <row r="11" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A11" t="s">
+        <v>10</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -2916,11 +2992,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Proceso_Solicitud</t>
-        </is>
+    <row r="12" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A12" t="s">
+        <v>11</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -3136,11 +3210,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Inicio_Proceso_AFP</t>
-        </is>
+    <row r="13" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A13" t="s">
+        <v>12</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -3356,11 +3428,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Formulario_Solicitud_Pension</t>
-        </is>
+    <row r="14" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A14" t="s">
+        <v>13</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -3576,11 +3646,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Certificado_de_Saldo</t>
-        </is>
+    <row r="15" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A15" t="s">
+        <v>14</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -3796,11 +3864,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Definicion_SCOMP</t>
-        </is>
+    <row r="16" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A16" t="s">
+        <v>15</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -4016,11 +4082,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Solicitud_Ofertas</t>
-        </is>
+    <row r="17" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A17" t="s">
+        <v>16</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -4236,11 +4300,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Certificado_Oferta</t>
-        </is>
+    <row r="18" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A18" t="s">
+        <v>17</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -4456,11 +4518,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Opciones_Post_Oferta</t>
-        </is>
+    <row r="19" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A19" t="s">
+        <v>18</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -4676,11 +4736,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Remate</t>
-        </is>
+    <row r="20" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A20" t="s">
+        <v>19</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -4896,11 +4954,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Evaluacion_Ofertas</t>
-        </is>
+    <row r="21" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A21" t="s">
+        <v>20</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -5116,11 +5172,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Acepta_Rechazo_Oferta</t>
-        </is>
+    <row r="22" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A22" t="s">
+        <v>21</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -5336,11 +5390,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Formulario_Seleccion_Modalidad</t>
-        </is>
+    <row r="23" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A23" t="s">
+        <v>22</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -5556,11 +5608,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Materializacion_Eleccion</t>
-        </is>
+    <row r="24" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A24" t="s">
+        <v>23</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -5776,11 +5826,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Causas_Finalizacion_Proceso</t>
-        </is>
+    <row r="25" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A25" t="s">
+        <v>24</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -5996,11 +6044,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Traslado_Fondos</t>
-        </is>
+    <row r="26" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A26" t="s">
+        <v>25</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -6216,11 +6262,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Inicio_Pagos</t>
-        </is>
+    <row r="27" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A27" t="s">
+        <v>26</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -6436,11 +6480,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Errores_Formularios</t>
-        </is>
+    <row r="28" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A28" t="s">
+        <v>27</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -6656,11 +6698,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Demora_Certificados</t>
-        </is>
+    <row r="29" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A29" t="s">
+        <v>28</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -6876,11 +6916,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Modalidades_Pensiones</t>
-        </is>
+    <row r="30" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A30" t="s">
+        <v>29</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -7096,11 +7134,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Comparacion_modalidades</t>
-        </is>
+    <row r="31" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A31" t="s">
+        <v>30</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -7316,11 +7352,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Expectativa_Vida</t>
-        </is>
+    <row r="32" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A32" t="s">
+        <v>31</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -7536,11 +7570,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Riesgo_Longevidad</t>
-        </is>
+    <row r="33" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A33" t="s">
+        <v>32</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -7756,11 +7788,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Riesgo_Rentabilidad</t>
-        </is>
+    <row r="34" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A34" t="s">
+        <v>33</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -7976,11 +8006,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Tasa_Interes_Tecnica_RP</t>
-        </is>
+    <row r="35" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A35" t="s">
+        <v>34</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -8196,11 +8224,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Tasa_Interes_RV</t>
-        </is>
+    <row r="36" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A36" t="s">
+        <v>35</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -8416,11 +8442,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Cambio_Modalidad</t>
-        </is>
+    <row r="37" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A37" t="s">
+        <v>36</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -8636,11 +8660,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Renta_Vitalicia</t>
-        </is>
+    <row r="38" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A38" t="s">
+        <v>37</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -8856,11 +8878,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Requisitos_RV</t>
-        </is>
+    <row r="39" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A39" t="s">
+        <v>38</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -9076,11 +9096,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Condiciones_Especiales_RV</t>
-        </is>
+    <row r="40" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A40" t="s">
+        <v>39</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -9296,11 +9314,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Periodo_Garantizado</t>
-        </is>
+    <row r="41" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A41" t="s">
+        <v>40</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -9516,11 +9532,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Clausula_Incremento_Sobrevivencia</t>
-        </is>
+    <row r="42" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A42" t="s">
+        <v>41</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -9736,11 +9750,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Aumento_Temporal</t>
-        </is>
+    <row r="43" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A43" t="s">
+        <v>42</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -9956,11 +9968,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Calculo_Renta_Vitalicia</t>
-        </is>
+    <row r="44" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A44" t="s">
+        <v>43</v>
       </c>
       <c r="B44">
         <v>0</v>
@@ -10176,11 +10186,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Retiro_Programado</t>
-        </is>
+    <row r="45" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A45" t="s">
+        <v>44</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -10396,11 +10404,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Requisitos_RP</t>
-        </is>
+    <row r="46" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A46" t="s">
+        <v>45</v>
       </c>
       <c r="B46">
         <v>0</v>
@@ -10616,11 +10622,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Calculo_Retiro_Programado</t>
-        </is>
+    <row r="47" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A47" t="s">
+        <v>46</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -10836,11 +10840,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>RVI_RP</t>
-        </is>
+    <row r="48" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A48" t="s">
+        <v>47</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -11056,11 +11058,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Requisitos_RVI_RP</t>
-        </is>
+    <row r="49" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A49" t="s">
+        <v>48</v>
       </c>
       <c r="B49">
         <v>0</v>
@@ -11276,11 +11276,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>RT_RVD</t>
-        </is>
+    <row r="50" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A50" t="s">
+        <v>49</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -11496,11 +11494,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Periodo_Diferimiento</t>
-        </is>
+    <row r="51" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A51" t="s">
+        <v>50</v>
       </c>
       <c r="B51">
         <v>0</v>
@@ -11716,11 +11712,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Requisitos_RT_RVD</t>
-        </is>
+    <row r="52" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A52" t="s">
+        <v>51</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -11936,11 +11930,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Calculo_Rentas_Combinadas</t>
-        </is>
+    <row r="53" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A53" t="s">
+        <v>52</v>
       </c>
       <c r="B53">
         <v>0</v>
@@ -12156,11 +12148,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Beneficiarios_Legales</t>
-        </is>
+    <row r="54" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A54" t="s">
+        <v>53</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -12376,11 +12366,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Declaracion_Beneficiarios</t>
-        </is>
+    <row r="55" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A55" t="s">
+        <v>54</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -12596,11 +12584,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Pension_Sobrevivencia</t>
-        </is>
+    <row r="56" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A56" t="s">
+        <v>55</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -12816,11 +12802,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Ejemplo_Calculo_Pension_Sobrevivencia</t>
-        </is>
+    <row r="57" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A57" t="s">
+        <v>56</v>
       </c>
       <c r="B57">
         <v>0</v>
@@ -13036,11 +13020,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Herencia</t>
-        </is>
+    <row r="58" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A58" t="s">
+        <v>57</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -13256,11 +13238,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Quien_Recibe_Herencia</t>
-        </is>
+    <row r="59" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A59" t="s">
+        <v>58</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -13476,11 +13456,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Como_Calcular_Herencia</t>
-        </is>
+    <row r="60" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A60" t="s">
+        <v>59</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -13696,11 +13674,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Definicion_APV</t>
-        </is>
+    <row r="61" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A61" t="s">
+        <v>60</v>
       </c>
       <c r="B61">
         <v>0</v>
@@ -13916,11 +13892,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Movilidad_Fondos_APV_Pension</t>
-        </is>
+    <row r="62" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A62" t="s">
+        <v>61</v>
       </c>
       <c r="B62">
         <v>0</v>
@@ -14136,11 +14110,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>ELD</t>
-        </is>
+    <row r="63" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A63" t="s">
+        <v>62</v>
       </c>
       <c r="B63">
         <v>0</v>
@@ -14356,11 +14328,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Calculo_ELD</t>
-        </is>
+    <row r="64" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A64" t="s">
+        <v>63</v>
       </c>
       <c r="B64">
         <v>0</v>
@@ -14576,11 +14546,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Tratamiento_Tributario_ELD</t>
-        </is>
+    <row r="65" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A65" t="s">
+        <v>64</v>
       </c>
       <c r="B65">
         <v>0</v>
@@ -14796,11 +14764,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Impacto_Pension_ELD</t>
-        </is>
+    <row r="66" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A66" t="s">
+        <v>65</v>
       </c>
       <c r="B66">
         <v>0</v>
@@ -15016,11 +14982,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Procedimiento_Retiro_ELD</t>
-        </is>
+    <row r="67" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A67" t="s">
+        <v>66</v>
       </c>
       <c r="B67">
         <v>0</v>
@@ -15236,11 +15200,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Asesores_Prev</t>
-        </is>
+    <row r="68" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A68" t="s">
+        <v>67</v>
       </c>
       <c r="B68">
         <v>0</v>
@@ -15456,11 +15418,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Comisiones_AFP</t>
-        </is>
+    <row r="69" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A69" t="s">
+        <v>68</v>
       </c>
       <c r="B69">
         <v>0</v>
@@ -15676,11 +15636,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Comisiones_Aseguradoras</t>
-        </is>
+    <row r="70" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A70" t="s">
+        <v>69</v>
       </c>
       <c r="B70">
         <v>0</v>
@@ -15896,11 +15854,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Impacto_Comisiones</t>
-        </is>
+    <row r="71" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A71" t="s">
+        <v>70</v>
       </c>
       <c r="B71">
         <v>0</v>
@@ -16116,11 +16072,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Falta_Claridad_Comisiones</t>
-        </is>
+    <row r="72" spans="1:72" x14ac:dyDescent="0.5">
+      <c r="A72" t="s">
+        <v>71</v>
       </c>
       <c r="B72">
         <v>0</v>

</xml_diff>